<commit_message>
Remove old orders page
</commit_message>
<xml_diff>
--- a/Lovely Oven Orders.xlsx
+++ b/Lovely Oven Orders.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/garybyatt/Documents/GitHub/Lovely Oven/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9145D5D-127E-3545-AACC-56EA68F11024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1BB6897-C795-9642-A471-A9EA81C82982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28740" windowHeight="18980" xr2:uid="{45BFCE97-D7BE-B145-B019-8CE646DEFA41}"/>
   </bookViews>
   <sheets>
     <sheet name="Fri 5th June" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,12 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
   <si>
     <t>Staff</t>
-  </si>
-  <si>
-    <t>Sam B</t>
   </si>
   <si>
     <t>Greg</t>
@@ -120,7 +117,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -130,6 +127,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -146,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -164,6 +167,7 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,7 +502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D3BA534-484A-1F44-91DA-F3FE4D7E1BB6}">
-  <dimension ref="B2:F13"/>
+  <dimension ref="B2:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.33203125" customWidth="1"/>
@@ -512,16 +516,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>7</v>
-      </c>
       <c r="F2" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.2">
@@ -529,13 +533,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
       </c>
       <c r="E3" s="6">
         <v>0.52083333333333337</v>
+      </c>
+      <c r="F3">
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.2">
@@ -543,30 +550,30 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="3">
-        <v>1</v>
-      </c>
-      <c r="E4" s="6">
-        <v>0.52083333333333337</v>
+        <v>2</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F4">
-        <v>70</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3">
-        <v>2</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>13</v>
+        <v>1</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0.52083333333333337</v>
       </c>
       <c r="F5">
         <v>70</v>
@@ -577,7 +584,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
@@ -585,16 +592,14 @@
       <c r="E6" s="6">
         <v>0.52083333333333337</v>
       </c>
-      <c r="F6">
-        <v>70</v>
-      </c>
+      <c r="F6" s="7"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
@@ -602,35 +607,21 @@
       <c r="E7" s="6">
         <v>0.52083333333333337</v>
       </c>
+      <c r="F7">
+        <v>70</v>
+      </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="3">
-        <v>1</v>
-      </c>
-      <c r="E8" s="6">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="F8">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="C13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="3">
-        <f>SUM(D3:D11)</f>
-        <v>7</v>
-      </c>
-      <c r="F13">
-        <f>SUM(F3:F8)</f>
-        <v>280</v>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="C12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="3">
+        <f>SUM(D3:D10)</f>
+        <v>6</v>
+      </c>
+      <c r="F12">
+        <f>SUM(F3:F7)</f>
+        <v>350</v>
       </c>
     </row>
   </sheetData>

</xml_diff>